<commit_message>
remove '!index' and '!key'
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE482087-28BF-A54C-9DB8-4D35A155316C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68186292-A074-B04B-A2B6-FC43F57D1FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="9" r:id="rId1"/>
@@ -1889,13 +1889,13 @@
     <t>#main.type=$&amp;key2=MAIN&amp;#main.condition=mainline_event</t>
   </si>
   <si>
-    <t>#define.value=$&amp;key1=TASK_TYPE</t>
-  </si>
-  <si>
     <t>item#item.id=$.id</t>
   </si>
   <si>
     <t>item#*.id=$.id</t>
+  </si>
+  <si>
+    <t>#define.value=$&amp;#define.key1=TASK_TYPE</t>
   </si>
 </sst>
 </file>
@@ -4159,7 +4159,7 @@
         <v>257</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
@@ -6538,10 +6538,10 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>261</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
add array type support
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1AA8E83-8F5F-CC4B-80EC-264645E6E92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1877A711-5BFE-48BD-9D6A-58D78B4ACC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="9" r:id="rId1"/>
@@ -1101,7 +1101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="269">
   <si>
     <t>id</t>
   </si>
@@ -1386,9 +1386,6 @@
   </si>
   <si>
     <t>int?</t>
-  </si>
-  <si>
-    <t>table?</t>
   </si>
   <si>
     <t>bool?</t>
@@ -1862,12 +1859,6 @@
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
-    <t>{200105}</t>
-  </si>
-  <si>
-    <t>{200106}</t>
-  </si>
-  <si>
     <t>[1]</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
@@ -1916,17 +1907,31 @@
   </si>
   <si>
     <t>参数类型</t>
+  </si>
+  <si>
+    <t>[200105]</t>
+  </si>
+  <si>
+    <t>[200106]</t>
+  </si>
+  <si>
+    <t>int[]?</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[]</t>
+    <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1955,7 +1960,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1975,7 +1980,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2128,7 +2133,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2193,12 +2198,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2261,7 +2260,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
   </cellStyles>
@@ -3187,150 +3186,150 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
-    <col min="5" max="5" width="45.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" customWidth="1"/>
-    <col min="8" max="9" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.625" customWidth="1"/>
+    <col min="3" max="3" width="16.625" customWidth="1"/>
+    <col min="4" max="4" width="25.625" customWidth="1"/>
+    <col min="5" max="5" width="45.875" customWidth="1"/>
+    <col min="6" max="6" width="18.625" customWidth="1"/>
+    <col min="8" max="9" width="12.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="42" t="s">
-        <v>254</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-    </row>
-    <row r="2" spans="1:9" ht="16">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A1" s="40" t="s">
+        <v>251</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+    </row>
+    <row r="2" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="F2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="33" t="s">
+      <c r="G2" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="34" t="s">
+      <c r="H2" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="34" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="16">
+      <c r="I2" s="32" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="33" t="s">
-        <v>264</v>
-      </c>
-      <c r="G3" s="33" t="s">
+      <c r="F3" s="31" t="s">
+        <v>261</v>
+      </c>
+      <c r="G3" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="34" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="16">
+      <c r="I3" s="32" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-    </row>
-    <row r="5" spans="1:9" ht="16">
+      <c r="B4" s="31" t="s">
+        <v>248</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+    </row>
+    <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="33" t="s">
-        <v>258</v>
-      </c>
-      <c r="G5" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="34" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="16">
+      <c r="B5" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="31" t="s">
+        <v>255</v>
+      </c>
+      <c r="G5" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33" t="s">
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-    </row>
-    <row r="7" spans="1:9" ht="16">
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+    </row>
+    <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="33" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -3348,18 +3347,18 @@
       <c r="G7" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="35" t="s">
+      <c r="H7" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="35" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="16">
+      <c r="I7" s="33" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="35"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="11" t="s">
         <v>19</v>
       </c>
@@ -3375,14 +3374,14 @@
       <c r="G8" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-    </row>
-    <row r="9" spans="1:9" ht="16">
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+    </row>
+    <row r="9" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A9" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="35"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="11" t="s">
         <v>19</v>
       </c>
@@ -3398,14 +3397,14 @@
       <c r="G9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-    </row>
-    <row r="10" spans="1:9" ht="16">
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+    </row>
+    <row r="10" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A10" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="35"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="11" t="s">
         <v>19</v>
       </c>
@@ -3421,14 +3420,14 @@
       <c r="G10" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-    </row>
-    <row r="11" spans="1:9" ht="16">
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+    </row>
+    <row r="11" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A11" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="35"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="11" t="s">
         <v>19</v>
       </c>
@@ -3444,14 +3443,14 @@
       <c r="G11" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-    </row>
-    <row r="12" spans="1:9" ht="16">
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
+    </row>
+    <row r="12" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A12" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="35"/>
+      <c r="B12" s="33"/>
       <c r="C12" s="11" t="s">
         <v>19</v>
       </c>
@@ -3467,14 +3466,14 @@
       <c r="G12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-    </row>
-    <row r="13" spans="1:9" ht="16">
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+    </row>
+    <row r="13" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A13" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="35"/>
+      <c r="B13" s="33"/>
       <c r="C13" s="11" t="s">
         <v>19</v>
       </c>
@@ -3490,14 +3489,14 @@
       <c r="G13" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-    </row>
-    <row r="14" spans="1:9" ht="16">
+      <c r="H13" s="33"/>
+      <c r="I13" s="33"/>
+    </row>
+    <row r="14" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A14" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="33" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -3515,16 +3514,16 @@
       <c r="G14" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="35" t="s">
+      <c r="H14" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="I14" s="35"/>
-    </row>
-    <row r="15" spans="1:9" ht="16">
+      <c r="I14" s="33"/>
+    </row>
+    <row r="15" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A15" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="35"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="11" t="s">
         <v>37</v>
       </c>
@@ -3540,14 +3539,14 @@
       <c r="G15" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-    </row>
-    <row r="16" spans="1:9" ht="16">
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+    </row>
+    <row r="16" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A16" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="35"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="11" t="s">
         <v>37</v>
       </c>
@@ -3563,14 +3562,14 @@
       <c r="G16" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-    </row>
-    <row r="17" spans="1:9" ht="16">
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+    </row>
+    <row r="17" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A17" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="35"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="11" t="s">
         <v>37</v>
       </c>
@@ -3586,14 +3585,14 @@
       <c r="G17" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-    </row>
-    <row r="18" spans="1:9" ht="16">
+      <c r="H17" s="33"/>
+      <c r="I17" s="33"/>
+    </row>
+    <row r="18" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A18" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="35"/>
+      <c r="B18" s="33"/>
       <c r="C18" s="11" t="s">
         <v>37</v>
       </c>
@@ -3609,14 +3608,14 @@
       <c r="G18" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-    </row>
-    <row r="19" spans="1:9" ht="16">
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+    </row>
+    <row r="19" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A19" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="35"/>
+      <c r="B19" s="33"/>
       <c r="C19" s="11" t="s">
         <v>37</v>
       </c>
@@ -3632,14 +3631,14 @@
       <c r="G19" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-    </row>
-    <row r="20" spans="1:9" ht="16">
+      <c r="H19" s="33"/>
+      <c r="I19" s="33"/>
+    </row>
+    <row r="20" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A20" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="35" t="s">
+      <c r="B20" s="33" t="s">
         <v>59</v>
       </c>
       <c r="C20" s="11" t="s">
@@ -3657,16 +3656,16 @@
       <c r="G20" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H20" s="35" t="s">
+      <c r="H20" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="I20" s="35"/>
-    </row>
-    <row r="21" spans="1:9" ht="16">
+      <c r="I20" s="33"/>
+    </row>
+    <row r="21" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A21" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="35"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="11" t="s">
         <v>60</v>
       </c>
@@ -3682,14 +3681,14 @@
       <c r="G21" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-    </row>
-    <row r="22" spans="1:9" ht="16">
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+    </row>
+    <row r="22" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A22" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="35"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="11" t="s">
         <v>60</v>
       </c>
@@ -3705,14 +3704,14 @@
       <c r="G22" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-    </row>
-    <row r="23" spans="1:9" ht="16">
+      <c r="H22" s="33"/>
+      <c r="I22" s="33"/>
+    </row>
+    <row r="23" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A23" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="35"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="11" t="s">
         <v>60</v>
       </c>
@@ -3728,31 +3727,31 @@
       <c r="G23" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-    </row>
-    <row r="24" spans="1:9" ht="16">
+      <c r="H23" s="33"/>
+      <c r="I23" s="33"/>
+    </row>
+    <row r="24" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A24" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="37" t="s">
+      <c r="B24" s="34"/>
+      <c r="C24" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="D24" s="37" t="s">
+      <c r="D24" s="35" t="s">
         <v>71</v>
       </c>
-      <c r="E24" s="37" t="s">
+      <c r="E24" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F24" s="37">
+      <c r="F24" s="35">
         <v>1023</v>
       </c>
-      <c r="G24" s="37" t="s">
+      <c r="G24" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3767,30 +3766,30 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{984B885C-48D0-4D9B-AAB3-39C5F463E278}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9" style="41"/>
+    <col min="1" max="1" width="9" style="39"/>
     <col min="2" max="2" width="32.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="49" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="44" t="s">
-        <v>255</v>
-      </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-    </row>
-    <row r="2" spans="1:5" ht="16">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="42" t="s">
+        <v>252</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
@@ -3802,7 +3801,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16">
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3819,7 +3818,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -3828,7 +3827,7 @@
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16">
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -3845,65 +3844,65 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="36" t="s">
         <v>235</v>
       </c>
-      <c r="C6" s="38" t="s">
+      <c r="D6" s="36" t="s">
         <v>236</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="E6" s="36" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
         <v>237</v>
       </c>
-      <c r="E6" s="38" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="41" t="s">
+      <c r="C7" s="37">
+        <v>1200</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="B7" t="s">
-        <v>238</v>
-      </c>
-      <c r="C7" s="39">
-        <v>1200</v>
-      </c>
-      <c r="D7" s="40" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="40" t="s">
+      <c r="B8" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>240</v>
-      </c>
-      <c r="C8" s="39">
+      <c r="C8" s="37">
         <v>3</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
       </c>
       <c r="E8" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>242</v>
-      </c>
-      <c r="C9" s="39">
+      <c r="C9" s="37">
         <f>7*3600</f>
         <v>25200</v>
       </c>
@@ -3911,17 +3910,17 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>244</v>
-      </c>
-      <c r="C10" s="39">
+      <c r="C10" s="37">
         <f>0.5*3600</f>
         <v>1800</v>
       </c>
@@ -3929,7 +3928,7 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -3945,26 +3944,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.1640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" style="9" customWidth="1"/>
-    <col min="3" max="4" width="15.1640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="26.83203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="8.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.1640625" style="8" customWidth="1"/>
-    <col min="8" max="8" width="23.1640625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="17.125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="17.875" style="9" customWidth="1"/>
+    <col min="3" max="4" width="15.125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="26.875" style="9" customWidth="1"/>
+    <col min="6" max="6" width="8.625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.125" style="9" customWidth="1"/>
+    <col min="8" max="8" width="23.125" style="9" customWidth="1"/>
     <col min="9" max="9" width="5" style="9" customWidth="1"/>
-    <col min="10" max="10" width="46.1640625" style="9" customWidth="1"/>
+    <col min="10" max="10" width="46.125" style="9" customWidth="1"/>
     <col min="11" max="11" width="31.5" style="9" customWidth="1"/>
     <col min="12" max="12" width="8" style="9" customWidth="1"/>
-    <col min="13" max="13" width="73.6640625" style="9" customWidth="1"/>
-    <col min="14" max="14" width="13.1640625" style="9" customWidth="1"/>
-    <col min="15" max="15" width="20.6640625" style="8" customWidth="1"/>
+    <col min="13" max="13" width="73.625" style="9" customWidth="1"/>
+    <col min="14" max="14" width="13.125" style="9" customWidth="1"/>
+    <col min="15" max="15" width="20.625" style="8" customWidth="1"/>
     <col min="16" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -3983,7 +3982,7 @@
       <c r="F1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="22" t="s">
+      <c r="G1" s="2" t="s">
         <v>77</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -4038,7 +4037,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="21" t="s">
         <v>22</v>
       </c>
@@ -4049,7 +4048,7 @@
         <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>11</v>
@@ -4057,26 +4056,26 @@
       <c r="F2" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="G2" s="22" t="s">
-        <v>95</v>
+      <c r="G2" s="2" t="s">
+        <v>267</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>94</v>
@@ -4112,7 +4111,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
         <v>12</v>
       </c>
@@ -4123,19 +4122,19 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="22"/>
+      <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>13</v>
@@ -4168,7 +4167,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" s="21" t="s">
         <v>14</v>
       </c>
@@ -4176,19 +4175,19 @@
         <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>13</v>
@@ -4197,11 +4196,11 @@
         <v>13</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="L4" s="2" t="s">
         <v>13</v>
       </c>
@@ -4209,7 +4208,7 @@
         <v>13</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="O4" s="12" t="s">
         <v>13</v>
@@ -4242,84 +4241,84 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>104</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>105</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>18</v>
       </c>
       <c r="E5" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="G5" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="J5" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="K5" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="L5" s="13" t="s">
         <v>111</v>
-      </c>
-      <c r="L5" s="13" t="s">
-        <v>112</v>
       </c>
       <c r="M5" s="13"/>
       <c r="N5" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="O5" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="P5" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="Q5" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="R5" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="R5" s="9" t="s">
+      <c r="S5" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="T5" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="S5" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="T5" s="9" t="s">
+      <c r="U5" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="V5" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="U5" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="V5" s="9" t="s">
+      <c r="W5" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="W5" s="9" t="s">
+      <c r="X5" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="X5" s="9" t="s">
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A6" s="22">
+        <v>1001</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" ht="17">
-      <c r="A6" s="24">
-        <v>1001</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>122</v>
       </c>
       <c r="C6" s="15">
         <v>1</v>
@@ -4327,14 +4326,16 @@
       <c r="D6" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="25" t="s">
-        <v>122</v>
+      <c r="E6" s="23" t="s">
+        <v>121</v>
       </c>
       <c r="F6" s="15">
         <f t="shared" ref="F6:F16" si="0">A7</f>
         <v>1002</v>
       </c>
-      <c r="G6" s="19"/>
+      <c r="G6" s="15" t="s">
+        <v>268</v>
+      </c>
       <c r="H6" s="16" t="s">
         <v>38</v>
       </c>
@@ -4342,7 +4343,7 @@
         <v>1</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K6" s="15" t="str">
         <f>"{"&amp;O6&amp;"}"</f>
@@ -4351,8 +4352,8 @@
       <c r="L6" s="15">
         <v>0</v>
       </c>
-      <c r="M6" s="29" t="s">
-        <v>124</v>
+      <c r="M6" s="27" t="s">
+        <v>123</v>
       </c>
       <c r="N6" s="9">
         <v>1</v>
@@ -4379,12 +4380,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
-      <c r="A7" s="24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A7" s="22">
         <v>1002</v>
       </c>
-      <c r="B7" s="25" t="s">
-        <v>125</v>
+      <c r="B7" s="23" t="s">
+        <v>124</v>
       </c>
       <c r="C7" s="15">
         <v>2</v>
@@ -4392,14 +4393,14 @@
       <c r="D7" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="25" t="s">
-        <v>125</v>
+      <c r="E7" s="23" t="s">
+        <v>124</v>
       </c>
       <c r="F7" s="15">
         <f t="shared" si="0"/>
         <v>1003</v>
       </c>
-      <c r="G7" s="19"/>
+      <c r="G7" s="15"/>
       <c r="H7" s="9" t="s">
         <v>38</v>
       </c>
@@ -4407,7 +4408,7 @@
         <v>1</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K7" s="15" t="str">
         <f t="shared" ref="K7:K9" si="1">"{"&amp;O7&amp;"}"</f>
@@ -4439,12 +4440,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="17">
-      <c r="A8" s="24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A8" s="22">
         <v>1003</v>
       </c>
-      <c r="B8" s="25" t="s">
-        <v>127</v>
+      <c r="B8" s="23" t="s">
+        <v>126</v>
       </c>
       <c r="C8" s="15">
         <v>3</v>
@@ -4452,8 +4453,8 @@
       <c r="D8" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="25" t="s">
-        <v>127</v>
+      <c r="E8" s="23" t="s">
+        <v>126</v>
       </c>
       <c r="F8" s="15">
         <f t="shared" si="0"/>
@@ -4466,7 +4467,7 @@
         <v>1</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K8" s="15" t="str">
         <f t="shared" si="1"/>
@@ -4504,12 +4505,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="17">
-      <c r="A9" s="24">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A9" s="22">
         <v>1014</v>
       </c>
-      <c r="B9" s="25" t="s">
-        <v>129</v>
+      <c r="B9" s="23" t="s">
+        <v>128</v>
       </c>
       <c r="C9" s="15">
         <v>4</v>
@@ -4517,15 +4518,15 @@
       <c r="D9" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="25" t="s">
-        <v>129</v>
+      <c r="E9" s="23" t="s">
+        <v>128</v>
       </c>
       <c r="F9" s="15">
         <f t="shared" si="0"/>
         <v>100301</v>
       </c>
-      <c r="G9" s="19" t="s">
-        <v>251</v>
+      <c r="G9" s="15" t="s">
+        <v>265</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>57</v>
@@ -4566,12 +4567,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
-      <c r="A10" s="24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A10" s="22">
         <v>100301</v>
       </c>
-      <c r="B10" s="25" t="s">
-        <v>130</v>
+      <c r="B10" s="23" t="s">
+        <v>129</v>
       </c>
       <c r="C10" s="15">
         <v>5</v>
@@ -4579,15 +4580,15 @@
       <c r="D10" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="25" t="s">
-        <v>130</v>
+      <c r="E10" s="23" t="s">
+        <v>129</v>
       </c>
       <c r="F10" s="15">
         <f t="shared" si="0"/>
         <v>100302</v>
       </c>
-      <c r="G10" s="19" t="s">
-        <v>252</v>
+      <c r="G10" s="15" t="s">
+        <v>266</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>38</v>
@@ -4596,7 +4597,7 @@
         <v>1</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K10" s="15" t="str">
         <f t="shared" ref="K10:K11" si="3">"{"&amp;O10&amp;"}"</f>
@@ -4605,8 +4606,8 @@
       <c r="L10" s="15">
         <v>0</v>
       </c>
-      <c r="M10" s="29" t="s">
-        <v>132</v>
+      <c r="M10" s="27" t="s">
+        <v>131</v>
       </c>
       <c r="N10" s="9">
         <v>1</v>
@@ -4636,12 +4637,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="17">
-      <c r="A11" s="24">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A11" s="22">
         <v>100302</v>
       </c>
-      <c r="B11" s="25" t="s">
-        <v>133</v>
+      <c r="B11" s="23" t="s">
+        <v>132</v>
       </c>
       <c r="C11" s="15">
         <v>6</v>
@@ -4649,14 +4650,14 @@
       <c r="D11" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="25" t="s">
-        <v>133</v>
+      <c r="E11" s="23" t="s">
+        <v>132</v>
       </c>
       <c r="F11" s="15">
         <f t="shared" si="0"/>
         <v>100303</v>
       </c>
-      <c r="G11" s="19"/>
+      <c r="G11" s="15"/>
       <c r="H11" s="16" t="s">
         <v>38</v>
       </c>
@@ -4664,7 +4665,7 @@
         <v>1</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K11" s="15" t="str">
         <f t="shared" si="3"/>
@@ -4696,48 +4697,48 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:24" s="20" customFormat="1" ht="17">
-      <c r="A12" s="26">
+    <row r="12" spans="1:24" s="20" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="24">
         <v>100303</v>
       </c>
-      <c r="B12" s="25" t="s">
-        <v>135</v>
+      <c r="B12" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="C12" s="15">
         <v>7</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="25" t="s">
-        <v>135</v>
+      <c r="E12" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="F12" s="15">
         <f t="shared" si="0"/>
         <v>100001</v>
       </c>
-      <c r="G12" s="28"/>
-      <c r="H12" s="30" t="s">
+      <c r="G12" s="26"/>
+      <c r="H12" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="I12" s="28">
+      <c r="I12" s="26">
         <v>1</v>
       </c>
-      <c r="J12" s="31" t="s">
-        <v>136</v>
-      </c>
-      <c r="K12" s="27" t="str">
+      <c r="J12" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="K12" s="25" t="str">
         <f t="shared" ref="K12:K17" si="5">"{"&amp;O12&amp;"}"</f>
         <v>{{10201,10}}</v>
       </c>
-      <c r="L12" s="27">
+      <c r="L12" s="25">
         <v>0</v>
       </c>
-      <c r="M12" s="27"/>
+      <c r="M12" s="25"/>
       <c r="N12" s="20">
         <v>1</v>
       </c>
-      <c r="O12" s="32" t="str">
+      <c r="O12" s="30" t="str">
         <f t="shared" ref="O12:O17" si="6">IF(P12="","","{"&amp;P12&amp;","&amp;Q12&amp;"}")&amp;IF(R12="","",",{"&amp;R12&amp;","&amp;S12&amp;"}")&amp;IF(T12="","",",{"&amp;T12&amp;","&amp;U12&amp;"}")</f>
         <v>{10201,10}</v>
       </c>
@@ -4756,12 +4757,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="17">
-      <c r="A13" s="24">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A13" s="22">
         <v>100001</v>
       </c>
-      <c r="B13" s="25" t="s">
-        <v>137</v>
+      <c r="B13" s="23" t="s">
+        <v>136</v>
       </c>
       <c r="C13" s="15">
         <v>8</v>
@@ -4769,14 +4770,14 @@
       <c r="D13" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="25" t="s">
-        <v>137</v>
+      <c r="E13" s="23" t="s">
+        <v>136</v>
       </c>
       <c r="F13" s="15">
         <f t="shared" si="0"/>
         <v>100002</v>
       </c>
-      <c r="G13" s="19"/>
+      <c r="G13" s="15"/>
       <c r="H13" s="16" t="s">
         <v>38</v>
       </c>
@@ -4784,7 +4785,7 @@
         <v>1</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K13" s="15" t="str">
         <f t="shared" ref="K13:K14" si="7">"{"&amp;O13&amp;"}"</f>
@@ -4816,12 +4817,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
-      <c r="A14" s="24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A14" s="22">
         <v>100002</v>
       </c>
-      <c r="B14" s="25" t="s">
-        <v>139</v>
+      <c r="B14" s="23" t="s">
+        <v>138</v>
       </c>
       <c r="C14" s="15">
         <v>9</v>
@@ -4829,14 +4830,14 @@
       <c r="D14" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="25" t="s">
-        <v>139</v>
+      <c r="E14" s="23" t="s">
+        <v>138</v>
       </c>
       <c r="F14" s="15">
         <f t="shared" si="0"/>
         <v>100003</v>
       </c>
-      <c r="G14" s="19"/>
+      <c r="G14" s="15"/>
       <c r="H14" s="9" t="s">
         <v>38</v>
       </c>
@@ -4844,7 +4845,7 @@
         <v>1</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K14" s="15" t="str">
         <f t="shared" si="7"/>
@@ -4876,12 +4877,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
-      <c r="A15" s="24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A15" s="22">
         <v>100003</v>
       </c>
-      <c r="B15" s="25" t="s">
-        <v>141</v>
+      <c r="B15" s="23" t="s">
+        <v>140</v>
       </c>
       <c r="C15" s="15">
         <v>10</v>
@@ -4889,14 +4890,14 @@
       <c r="D15" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="25" t="s">
-        <v>141</v>
+      <c r="E15" s="23" t="s">
+        <v>140</v>
       </c>
       <c r="F15" s="15">
         <f t="shared" si="0"/>
         <v>100304</v>
       </c>
-      <c r="G15" s="19"/>
+      <c r="G15" s="15"/>
       <c r="H15" s="9" t="s">
         <v>38</v>
       </c>
@@ -4904,7 +4905,7 @@
         <v>1</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K15" s="15" t="str">
         <f t="shared" ref="K15" si="9">"{"&amp;O15&amp;"}"</f>
@@ -4913,8 +4914,8 @@
       <c r="L15" s="15">
         <v>0</v>
       </c>
-      <c r="M15" s="29" t="s">
-        <v>143</v>
+      <c r="M15" s="27" t="s">
+        <v>142</v>
       </c>
       <c r="N15" s="9">
         <v>1</v>
@@ -4938,12 +4939,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="17">
-      <c r="A16" s="24">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A16" s="22">
         <v>100304</v>
       </c>
-      <c r="B16" s="25" t="s">
-        <v>144</v>
+      <c r="B16" s="23" t="s">
+        <v>143</v>
       </c>
       <c r="C16" s="15">
         <v>11</v>
@@ -4951,14 +4952,14 @@
       <c r="D16" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="25" t="s">
-        <v>144</v>
+      <c r="E16" s="23" t="s">
+        <v>143</v>
       </c>
       <c r="F16" s="15">
         <f t="shared" si="0"/>
         <v>1013</v>
       </c>
-      <c r="G16" s="19"/>
+      <c r="G16" s="15"/>
       <c r="H16" s="16" t="s">
         <v>38</v>
       </c>
@@ -4966,7 +4967,7 @@
         <v>1</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K16" s="15" t="str">
         <f t="shared" si="5"/>
@@ -4998,12 +4999,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="17">
-      <c r="A17" s="24">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A17" s="22">
         <v>1013</v>
       </c>
-      <c r="B17" s="25" t="s">
-        <v>146</v>
+      <c r="B17" s="23" t="s">
+        <v>145</v>
       </c>
       <c r="C17" s="15">
         <v>12</v>
@@ -5011,11 +5012,11 @@
       <c r="D17" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="25" t="s">
-        <v>146</v>
+      <c r="E17" s="23" t="s">
+        <v>145</v>
       </c>
       <c r="F17" s="15"/>
-      <c r="G17" s="19"/>
+      <c r="G17" s="15"/>
       <c r="H17" s="16" t="s">
         <v>54</v>
       </c>
@@ -5023,7 +5024,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="19" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K17" s="15" t="str">
         <f t="shared" si="5"/>
@@ -5070,27 +5071,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.1640625" style="9" customWidth="1"/>
-    <col min="2" max="3" width="17.83203125" style="9" customWidth="1"/>
-    <col min="4" max="5" width="15.1640625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="17.125" style="9" customWidth="1"/>
+    <col min="2" max="3" width="17.875" style="9" customWidth="1"/>
+    <col min="4" max="5" width="15.125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="19.875" style="9" customWidth="1"/>
     <col min="7" max="7" width="28" style="9" customWidth="1"/>
-    <col min="8" max="8" width="15.1640625" style="9" customWidth="1"/>
-    <col min="9" max="9" width="23.1640625" style="9" customWidth="1"/>
-    <col min="10" max="10" width="16.1640625" style="9" customWidth="1"/>
-    <col min="11" max="11" width="63.1640625" style="9" customWidth="1"/>
-    <col min="12" max="12" width="8.83203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.1640625" style="9" customWidth="1"/>
-    <col min="14" max="14" width="13.1640625" style="9" customWidth="1"/>
+    <col min="8" max="8" width="15.125" style="9" customWidth="1"/>
+    <col min="9" max="9" width="23.125" style="9" customWidth="1"/>
+    <col min="10" max="10" width="16.125" style="9" customWidth="1"/>
+    <col min="11" max="11" width="63.125" style="9" customWidth="1"/>
+    <col min="12" max="12" width="8.875" style="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.125" style="9" customWidth="1"/>
+    <col min="14" max="14" width="13.125" style="9" customWidth="1"/>
     <col min="15" max="15" width="9" style="9"/>
-    <col min="16" max="16" width="13.1640625" style="9" customWidth="1"/>
+    <col min="16" max="16" width="13.125" style="9" customWidth="1"/>
     <col min="17" max="17" width="11" style="9" customWidth="1"/>
     <col min="18" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5098,7 +5099,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>73</v>
@@ -5107,7 +5108,7 @@
         <v>74</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>75</v>
@@ -5125,7 +5126,7 @@
         <v>8</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>80</v>
@@ -5161,7 +5162,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -5175,7 +5176,7 @@
         <v>22</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>11</v>
@@ -5190,16 +5191,16 @@
         <v>11</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>11</v>
@@ -5232,7 +5233,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -5243,7 +5244,7 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -5253,13 +5254,13 @@
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>13</v>
@@ -5284,7 +5285,7 @@
       </c>
       <c r="X3" s="1"/>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -5307,7 +5308,7 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>13</v>
@@ -5322,7 +5323,7 @@
         <v>13</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>13</v>
@@ -5356,82 +5357,82 @@
       </c>
       <c r="X4" s="12"/>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>104</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>105</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G5" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="K5" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="L5" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="M5" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="L5" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="M5" s="13" t="s">
+      <c r="N5" s="13" t="s">
         <v>111</v>
-      </c>
-      <c r="N5" s="13" t="s">
-        <v>112</v>
       </c>
       <c r="O5" s="13"/>
       <c r="P5" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q5" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="Q5" s="8" t="s">
+      <c r="R5" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="R5" s="9" t="s">
+      <c r="S5" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="S5" s="9" t="s">
+      <c r="T5" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="T5" s="9" t="s">
+      <c r="U5" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="V5" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="U5" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="V5" s="9" t="s">
-        <v>118</v>
-      </c>
       <c r="W5" s="9" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <f t="shared" ref="A6:A16" si="0">200000+C6*100+D6</f>
         <v>200101</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C6" s="6">
         <f>COUNTIF($D$6:D6,1)</f>
@@ -5444,7 +5445,7 @@
         <v>24</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G6" s="6" t="str">
         <f>"支线·"&amp;F6</f>
@@ -5458,10 +5459,10 @@
         <v>0</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M6" s="15" t="str">
         <f t="shared" ref="M6:M16" si="1">"{"&amp;Q6&amp;"}"</f>
@@ -5485,13 +5486,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <f t="shared" si="0"/>
         <v>200102</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C7" s="6">
         <v>1</v>
@@ -5503,7 +5504,7 @@
         <v>24</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G7" s="6" t="str">
         <f t="shared" ref="G7:G16" si="3">"支线·"&amp;F7</f>
@@ -5520,7 +5521,7 @@
         <v>53</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M7" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5544,13 +5545,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <f t="shared" si="0"/>
         <v>200103</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C8" s="6">
         <v>1</v>
@@ -5562,7 +5563,7 @@
         <v>24</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G8" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5579,10 +5580,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M8" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5606,13 +5607,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <f t="shared" si="0"/>
         <v>200104</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C9" s="6">
         <v>1</v>
@@ -5624,7 +5625,7 @@
         <v>24</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G9" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5638,10 +5639,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M9" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5665,13 +5666,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <f t="shared" si="0"/>
         <v>200105</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C10" s="6">
         <v>1</v>
@@ -5683,7 +5684,7 @@
         <v>24</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G10" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5697,10 +5698,10 @@
         <v>0</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M10" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5724,13 +5725,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <f t="shared" si="0"/>
         <v>200106</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C11" s="6">
         <v>1</v>
@@ -5742,7 +5743,7 @@
         <v>24</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G11" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5756,10 +5757,10 @@
         <v>0</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M11" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5783,13 +5784,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
         <f t="shared" si="0"/>
         <v>200107</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C12" s="6">
         <v>1</v>
@@ -5801,7 +5802,7 @@
         <v>24</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G12" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5815,10 +5816,10 @@
         <v>0</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M12" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5842,13 +5843,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
         <f t="shared" si="0"/>
         <v>200201</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C13" s="6">
         <v>2</v>
@@ -5860,7 +5861,7 @@
         <v>24</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G13" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5877,10 +5878,10 @@
         <v>0</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M13" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5904,13 +5905,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" s="9">
         <f t="shared" si="0"/>
         <v>200202</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C14" s="6">
         <v>2</v>
@@ -5922,7 +5923,7 @@
         <v>24</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G14" s="6" t="str">
         <f t="shared" si="3"/>
@@ -5939,10 +5940,10 @@
         <v>0</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M14" s="15" t="str">
         <f t="shared" si="1"/>
@@ -5966,13 +5967,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <f t="shared" si="0"/>
         <v>200203</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C15" s="6">
         <v>2</v>
@@ -5984,7 +5985,7 @@
         <v>24</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G15" s="6" t="str">
         <f t="shared" si="3"/>
@@ -6001,10 +6002,10 @@
         <v>0</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M15" s="15" t="str">
         <f t="shared" si="1"/>
@@ -6028,13 +6029,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" s="9">
         <f t="shared" si="0"/>
         <v>200204</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C16" s="6">
         <v>2</v>
@@ -6046,7 +6047,7 @@
         <v>24</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G16" s="6" t="str">
         <f t="shared" si="3"/>
@@ -6060,10 +6061,10 @@
         <v>0</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M16" s="15" t="str">
         <f t="shared" si="1"/>
@@ -6101,16 +6102,16 @@
     <tabColor theme="5" tint="0.39915158543656726"/>
   </sheetPr>
   <dimension ref="A1:I19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="17.1640625" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" style="9" customWidth="1"/>
-    <col min="4" max="7" width="17.1640625" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" customWidth="1"/>
-    <col min="9" max="9" width="13.1640625" style="9" customWidth="1"/>
+    <col min="1" max="2" width="17.125" customWidth="1"/>
+    <col min="3" max="3" width="15.125" style="9" customWidth="1"/>
+    <col min="4" max="7" width="17.125" customWidth="1"/>
+    <col min="8" max="8" width="20.125" customWidth="1"/>
+    <col min="9" max="9" width="13.125" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6139,7 +6140,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6159,16 +6160,16 @@
         <v>11</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6179,17 +6180,17 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6212,47 +6213,47 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G5" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="C6" s="6">
         <v>1</v>
@@ -6261,27 +6262,27 @@
         <v>4</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>180</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>181</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>182</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>183</v>
       </c>
       <c r="C7" s="6">
         <v>2</v>
@@ -6290,27 +6291,27 @@
         <v>4</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>185</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>186</v>
       </c>
       <c r="I7" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>187</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>188</v>
       </c>
       <c r="C8" s="6">
         <v>3</v>
@@ -6319,27 +6320,27 @@
         <v>4</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>190</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="I8" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>192</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>193</v>
       </c>
       <c r="C9" s="6">
         <v>4</v>
@@ -6348,22 +6349,22 @@
         <v>4</v>
       </c>
       <c r="E9" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="G9" s="6" t="s">
+      <c r="H9" s="6" t="s">
         <v>195</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>196</v>
       </c>
       <c r="I9" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
@@ -6374,7 +6375,7 @@
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
@@ -6385,7 +6386,7 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -6396,7 +6397,7 @@
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -6407,7 +6408,7 @@
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
@@ -6418,7 +6419,7 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="4"/>
       <c r="B15" s="5"/>
       <c r="C15" s="6"/>
@@ -6429,7 +6430,7 @@
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="4"/>
       <c r="B16" s="5"/>
       <c r="C16" s="6"/>
@@ -6440,7 +6441,7 @@
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="4"/>
       <c r="B17" s="5"/>
       <c r="C17" s="6"/>
@@ -6451,7 +6452,7 @@
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
       <c r="B18" s="5"/>
       <c r="C18" s="6"/>
@@ -6462,7 +6463,7 @@
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="4"/>
       <c r="B19" s="5"/>
       <c r="C19" s="6"/>
@@ -6486,17 +6487,17 @@
     <tabColor theme="5" tint="0.39915158543656726"/>
   </sheetPr>
   <dimension ref="A1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="17.1640625" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="17.125" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="17.1640625" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" style="9" customWidth="1"/>
-    <col min="4" max="7" width="17.1640625" customWidth="1"/>
-    <col min="8" max="9" width="25.6640625" customWidth="1"/>
-    <col min="10" max="10" width="13.1640625" style="9" customWidth="1"/>
-    <col min="11" max="16377" width="17.1640625" customWidth="1"/>
+    <col min="1" max="2" width="17.125" customWidth="1"/>
+    <col min="3" max="3" width="15.125" style="9" customWidth="1"/>
+    <col min="4" max="7" width="17.125" customWidth="1"/>
+    <col min="8" max="9" width="25.625" customWidth="1"/>
+    <col min="10" max="10" width="13.125" style="9" customWidth="1"/>
+    <col min="11" max="16377" width="17.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6522,13 +6523,13 @@
         <v>80</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6548,19 +6549,19 @@
         <v>11</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6571,18 +6572,18 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6605,53 +6606,53 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G5" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="J5" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="I5" s="7" t="s">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="J5" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>199</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>200</v>
       </c>
       <c r="C6" s="6">
         <v>1</v>
@@ -6669,21 +6670,21 @@
         <v>45</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J6" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>202</v>
       </c>
       <c r="C7" s="6">
         <v>2</v>
@@ -6692,30 +6693,30 @@
         <v>5</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J7" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="C8" s="6">
         <v>3</v>
@@ -6724,30 +6725,30 @@
         <v>5</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J8" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>209</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>210</v>
       </c>
       <c r="C9" s="6">
         <v>4</v>
@@ -6756,25 +6757,25 @@
         <v>5</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J9" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
@@ -6786,7 +6787,7 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
@@ -6798,7 +6799,7 @@
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -6810,7 +6811,7 @@
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -6822,7 +6823,7 @@
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
@@ -6834,19 +6835,19 @@
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="J15" s="6"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="J16" s="6"/>
     </row>
-    <row r="17" spans="10:10">
+    <row r="17" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J17" s="6"/>
     </row>
-    <row r="18" spans="10:10">
+    <row r="18" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J18" s="6"/>
     </row>
-    <row r="19" spans="10:10">
+    <row r="19" spans="10:10" x14ac:dyDescent="0.35">
       <c r="J19" s="6"/>
     </row>
   </sheetData>
@@ -6859,18 +6860,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="10.625" customWidth="1"/>
     <col min="5" max="5" width="29" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="9" max="9" width="35.6640625" customWidth="1"/>
-    <col min="10" max="10" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.875" customWidth="1"/>
+    <col min="7" max="7" width="16.625" customWidth="1"/>
+    <col min="9" max="9" width="35.625" customWidth="1"/>
+    <col min="10" max="10" width="21.875" customWidth="1"/>
     <col min="12" max="12" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16">
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6908,7 +6909,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16">
+    <row r="2" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6931,22 +6932,22 @@
         <v>11</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="16">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6958,19 +6959,19 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="16">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6987,7 +6988,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -6999,7 +7000,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>13</v>
@@ -7008,50 +7009,50 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16">
+    <row r="5" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="K5" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="K5" s="7" t="s">
-        <v>112</v>
-      </c>
       <c r="L5" s="7" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="16">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>214</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>215</v>
       </c>
       <c r="C6" s="6">
         <v>2</v>
@@ -7060,7 +7061,7 @@
         <v>7</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6" t="s">
@@ -7068,24 +7069,24 @@
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>217</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>218</v>
       </c>
       <c r="K6" s="6">
         <v>0</v>
       </c>
       <c r="L6" s="8" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" ht="16">
-      <c r="A7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>220</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>221</v>
       </c>
       <c r="C7" s="6">
         <v>3</v>
@@ -7094,7 +7095,7 @@
         <v>7</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6" t="s">
@@ -7102,24 +7103,24 @@
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="J7" s="6" t="s">
         <v>222</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>223</v>
       </c>
       <c r="K7" s="6">
         <v>0</v>
       </c>
       <c r="L7" s="8" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" ht="16">
-      <c r="A8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>225</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>226</v>
       </c>
       <c r="C8" s="6">
         <v>4</v>
@@ -7128,7 +7129,7 @@
         <v>7</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6" t="s">
@@ -7136,24 +7137,24 @@
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="J8" s="6" t="s">
         <v>227</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>228</v>
       </c>
       <c r="K8" s="6">
         <v>0</v>
       </c>
       <c r="L8" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" ht="16">
-      <c r="A9" s="4" t="s">
-        <v>230</v>
-      </c>
       <c r="B9" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C9" s="6">
         <v>5</v>
@@ -7162,7 +7163,7 @@
         <v>7</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6" t="s">
@@ -7170,16 +7171,16 @@
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K9" s="6">
         <v>0</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add example for stringify rule
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F93D561-9D48-44CC-A724-6B5D31344B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718CF2AC-EFC2-455B-8CF6-1B8D933B94F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-15" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32100" yWindow="1425" windowWidth="28395" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="9" r:id="rId1"/>
@@ -1863,10 +1863,6 @@
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
-    <t>@define</t>
-    <phoneticPr fontId="8" type="noConversion"/>
-  </si>
-  <si>
     <t>@config</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
@@ -1924,6 +1920,10 @@
   </si>
   <si>
     <t>task#*.id&amp;type=MAIN</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>@define;@stringify(task)</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
@@ -3202,7 +3202,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="40" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
@@ -3256,7 +3256,7 @@
         <v>10</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G3" s="31" t="s">
         <v>11</v>
@@ -3300,7 +3300,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="31" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G5" s="31" t="s">
         <v>13</v>
@@ -3781,7 +3781,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="42" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -4052,7 +4052,7 @@
         <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>11</v>
@@ -4061,7 +4061,7 @@
         <v>94</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>11</v>
@@ -4179,19 +4179,19 @@
         <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>254</v>
-      </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>13</v>
@@ -4338,7 +4338,7 @@
         <v>1002</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H6" s="16" t="s">
         <v>38</v>
@@ -4530,7 +4530,7 @@
         <v>100301</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>57</v>
@@ -4592,7 +4592,7 @@
         <v>100302</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>38</v>
@@ -5130,7 +5130,7 @@
         <v>8</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>80</v>
@@ -5180,7 +5180,7 @@
         <v>22</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>11</v>
@@ -5198,7 +5198,7 @@
         <v>95</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>11</v>
@@ -5327,7 +5327,7 @@
         <v>13</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>13</v>
@@ -5396,7 +5396,7 @@
         <v>109</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M5" s="13" t="s">
         <v>110</v>
@@ -6610,10 +6610,10 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>256</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>257</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>13</v>

</xml_diff>